<commit_message>
7th commit working for 2023 PDF PARTIAL
</commit_message>
<xml_diff>
--- a/nirf_scores.xlsx
+++ b/nirf_scores.xlsx
@@ -433,15 +433,47 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:AL2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="11" customWidth="1" min="30" max="30"/>
+    <col width="11" customWidth="1" min="31" max="31"/>
+    <col width="10" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="10" customWidth="1" min="34" max="34"/>
+    <col width="10" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="11" customWidth="1" min="37" max="37"/>
+    <col width="10" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -467,10 +499,170 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>SS Score</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>FSR Score</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>FQE Score</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>FRU Score</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>PU Score</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>QP Score</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>IPR Score</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>FPPP Score</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>GPH Score</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>GUE Score</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>MS Score</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>GPHD Score</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>RD Score</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>WD Score</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>ESCS Score</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>PCS Score</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
           <t>PR Score</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>SS Total</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>FSR Total</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>FQE Total</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>FRU Total</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>PU Total</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>QP Total</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>IPR Total</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>FPPP Total</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>GPH Total</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>GUE Total</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>MS Total</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>GPHD Total</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>RD Total</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>WD Total</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>ESCS Total</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>PCS Total</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>PR Total</t>
         </is>
@@ -484,27 +676,187 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>medical</t>
+          <t>engineering</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>PSG INSTITUTE OF MEDICAL SCIENCES &amp; RESEARCH (Inst. Code - 012), COIMBATORE</t>
+          <t>Rajiv Gandhi Institute of Petroleum Technology</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>IR-D-C-45515</t>
+          <t>IR-E-U-0535</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8.00</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>6.82</t>
+          <t>29.47</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>18.57</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>20.64</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>3.02</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>7.11</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>0.00</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>2.43</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>37.12</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>15.00</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>13.87</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>18.19</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>13.02</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>3.36</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+      <c r="W2" s="2" t="inlineStr">
+        <is>
+          <t>30.00</t>
+        </is>
+      </c>
+      <c r="X2" s="2" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+      <c r="Y2" s="2" t="inlineStr">
+        <is>
+          <t>30.00</t>
+        </is>
+      </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>35.00</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>15.00</t>
+        </is>
+      </c>
+      <c r="AC2" s="2" t="inlineStr">
+        <is>
+          <t>10.00</t>
+        </is>
+      </c>
+      <c r="AD2" s="2" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="AE2" s="2" t="inlineStr">
+        <is>
+          <t>15.00</t>
+        </is>
+      </c>
+      <c r="AF2" s="2" t="inlineStr">
+        <is>
+          <t>25.00</t>
+        </is>
+      </c>
+      <c r="AG2" s="2" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>30.00</t>
+        </is>
+      </c>
+      <c r="AI2" s="2" t="inlineStr">
+        <is>
+          <t>30.00</t>
+        </is>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+      <c r="AK2" s="2" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
+        <is>
+          <t>100.00</t>
         </is>
       </c>
     </row>

</xml_diff>